<commit_message>
Complete audit fixes and synchronize bilingual portfolio materials
</commit_message>
<xml_diff>
--- a/data/raw/clients_raw.xlsx
+++ b/data/raw/clients_raw.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clients_raw" sheetId="1" r:id="R8d8ab5a84140441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clients_raw" sheetId="1" r:id="R4b02e14b119b41e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,6 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
@@ -63,7 +66,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -82,6 +85,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -342,7 +348,7 @@
       <x:c r="D2" s="9" t="str">
         <x:v>Казань</x:v>
       </x:c>
-      <x:c r="E2" s="9" t="n">
+      <x:c r="E2" s="10" t="n">
         <x:v>45472</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
@@ -362,7 +368,7 @@
       <x:c r="D3" s="9" t="str">
         <x:v>Казань</x:v>
       </x:c>
-      <x:c r="E3" s="9" t="n">
+      <x:c r="E3" s="10" t="n">
         <x:v>45513</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
@@ -382,7 +388,7 @@
       <x:c r="D4" s="9" t="str">
         <x:v>Москва</x:v>
       </x:c>
-      <x:c r="E4" s="9" t="n">
+      <x:c r="E4" s="10" t="n">
         <x:v>45465</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
@@ -402,7 +408,7 @@
       <x:c r="D5" s="9" t="str">
         <x:v>Самара</x:v>
       </x:c>
-      <x:c r="E5" s="9" t="n">
+      <x:c r="E5" s="10" t="n">
         <x:v>45299</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
@@ -420,7 +426,7 @@
       <x:c r="D6" s="9" t="str">
         <x:v>Краснодар</x:v>
       </x:c>
-      <x:c r="E6" s="9" t="n">
+      <x:c r="E6" s="10" t="n">
         <x:v>45872</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
@@ -440,7 +446,7 @@
       <x:c r="D7" s="9" t="str">
         <x:v>Москва</x:v>
       </x:c>
-      <x:c r="E7" s="9" t="n">
+      <x:c r="E7" s="10" t="n">
         <x:v>45846</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
@@ -460,7 +466,7 @@
       <x:c r="D8" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E8" s="9" t="n">
+      <x:c r="E8" s="10" t="n">
         <x:v>45601</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
@@ -480,7 +486,7 @@
       <x:c r="D9" s="9" t="str">
         <x:v>Екатеринбург</x:v>
       </x:c>
-      <x:c r="E9" s="9" t="n">
+      <x:c r="E9" s="10" t="n">
         <x:v>45750</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
@@ -500,7 +506,7 @@
       <x:c r="D10" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E10" s="9" t="n">
+      <x:c r="E10" s="10" t="n">
         <x:v>45304</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
@@ -520,7 +526,7 @@
       <x:c r="D11" s="9" t="str">
         <x:v>Москва</x:v>
       </x:c>
-      <x:c r="E11" s="9" t="n">
+      <x:c r="E11" s="10" t="n">
         <x:v>45313</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
@@ -540,7 +546,7 @@
       <x:c r="D12" s="9" t="str">
         <x:v>Краснодар</x:v>
       </x:c>
-      <x:c r="E12" s="9" t="n">
+      <x:c r="E12" s="10" t="n">
         <x:v>45995</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
@@ -560,7 +566,7 @@
       <x:c r="D13" s="9" t="str">
         <x:v>Екатеринбург</x:v>
       </x:c>
-      <x:c r="E13" s="9" t="n">
+      <x:c r="E13" s="10" t="n">
         <x:v>45413</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
@@ -580,7 +586,7 @@
       <x:c r="D14" s="9" t="str">
         <x:v>Москва</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="n">
+      <x:c r="E14" s="10" t="n">
         <x:v>45657</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str">
@@ -600,7 +606,7 @@
       <x:c r="D15" s="9" t="str">
         <x:v>Самара</x:v>
       </x:c>
-      <x:c r="E15" s="9" t="n">
+      <x:c r="E15" s="10" t="n">
         <x:v>45553</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str">
@@ -620,7 +626,7 @@
       <x:c r="D16" s="9" t="str">
         <x:v>Казань</x:v>
       </x:c>
-      <x:c r="E16" s="9" t="n">
+      <x:c r="E16" s="10" t="n">
         <x:v>45732</x:v>
       </x:c>
       <x:c r="F16" s="9" t="str">
@@ -640,7 +646,7 @@
       <x:c r="D17" s="9" t="str">
         <x:v>Краснодар</x:v>
       </x:c>
-      <x:c r="E17" s="9" t="n">
+      <x:c r="E17" s="10" t="n">
         <x:v>45998</x:v>
       </x:c>
       <x:c r="F17" s="9" t="str">
@@ -660,7 +666,7 @@
       <x:c r="D18" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E18" s="9" t="n">
+      <x:c r="E18" s="10" t="n">
         <x:v>45923</x:v>
       </x:c>
       <x:c r="F18" s="9" t="str">
@@ -678,7 +684,7 @@
         <x:v>7700000018</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str"/>
-      <x:c r="E19" s="9" t="n">
+      <x:c r="E19" s="10" t="n">
         <x:v>45555</x:v>
       </x:c>
       <x:c r="F19" s="9" t="str">
@@ -698,7 +704,7 @@
       <x:c r="D20" s="9" t="str">
         <x:v>Самара</x:v>
       </x:c>
-      <x:c r="E20" s="9" t="n">
+      <x:c r="E20" s="10" t="n">
         <x:v>45603</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
@@ -718,7 +724,7 @@
       <x:c r="D21" s="9" t="str">
         <x:v>Краснодар</x:v>
       </x:c>
-      <x:c r="E21" s="9" t="n">
+      <x:c r="E21" s="10" t="n">
         <x:v>45296</x:v>
       </x:c>
       <x:c r="F21" s="9" t="str">
@@ -738,7 +744,7 @@
       <x:c r="D22" s="9" t="str">
         <x:v>Екатеринбург</x:v>
       </x:c>
-      <x:c r="E22" s="9" t="n">
+      <x:c r="E22" s="10" t="n">
         <x:v>45926</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
@@ -758,7 +764,7 @@
       <x:c r="D23" s="9" t="str">
         <x:v>Казань</x:v>
       </x:c>
-      <x:c r="E23" s="9" t="n">
+      <x:c r="E23" s="10" t="n">
         <x:v>45381</x:v>
       </x:c>
       <x:c r="F23" s="9" t="str">
@@ -778,7 +784,7 @@
       <x:c r="D24" s="9" t="str">
         <x:v>Екатеринбург</x:v>
       </x:c>
-      <x:c r="E24" s="9" t="n">
+      <x:c r="E24" s="10" t="n">
         <x:v>45994</x:v>
       </x:c>
       <x:c r="F24" s="9" t="str">
@@ -798,7 +804,7 @@
       <x:c r="D25" s="9" t="str">
         <x:v>Екатеринбург</x:v>
       </x:c>
-      <x:c r="E25" s="9" t="n">
+      <x:c r="E25" s="10" t="n">
         <x:v>45514</x:v>
       </x:c>
       <x:c r="F25" s="9" t="str">
@@ -818,7 +824,7 @@
       <x:c r="D26" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E26" s="9" t="str"/>
+      <x:c r="E26" s="10" t="str"/>
       <x:c r="F26" s="9" t="str">
         <x:v>B2C</x:v>
       </x:c>
@@ -836,7 +842,7 @@
       <x:c r="D27" s="9" t="str">
         <x:v>Самара</x:v>
       </x:c>
-      <x:c r="E27" s="9" t="n">
+      <x:c r="E27" s="10" t="n">
         <x:v>45509</x:v>
       </x:c>
       <x:c r="F27" s="9" t="str">
@@ -856,7 +862,7 @@
       <x:c r="D28" s="9" t="str">
         <x:v>Самара</x:v>
       </x:c>
-      <x:c r="E28" s="9" t="n">
+      <x:c r="E28" s="10" t="n">
         <x:v>45549</x:v>
       </x:c>
       <x:c r="F28" s="9" t="str">
@@ -876,7 +882,7 @@
       <x:c r="D29" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E29" s="9" t="n">
+      <x:c r="E29" s="10" t="n">
         <x:v>45502</x:v>
       </x:c>
       <x:c r="F29" s="9" t="str">
@@ -896,7 +902,7 @@
       <x:c r="D30" s="9" t="str">
         <x:v>Новосибирск</x:v>
       </x:c>
-      <x:c r="E30" s="9" t="n">
+      <x:c r="E30" s="10" t="n">
         <x:v>45370</x:v>
       </x:c>
       <x:c r="F30" s="9" t="str">
@@ -916,7 +922,7 @@
       <x:c r="D31" s="9" t="str">
         <x:v>Краснодар</x:v>
       </x:c>
-      <x:c r="E31" s="9" t="n">
+      <x:c r="E31" s="10" t="n">
         <x:v>45540</x:v>
       </x:c>
       <x:c r="F31" s="9" t="str">
@@ -936,7 +942,7 @@
       <x:c r="D32" s="9" t="str">
         <x:v>Москва</x:v>
       </x:c>
-      <x:c r="E32" s="9" t="n">
+      <x:c r="E32" s="10" t="n">
         <x:v>45619</x:v>
       </x:c>
       <x:c r="F32" s="9" t="str">
@@ -956,7 +962,7 @@
       <x:c r="D33" s="9" t="str">
         <x:v>Москва</x:v>
       </x:c>
-      <x:c r="E33" s="9" t="n">
+      <x:c r="E33" s="10" t="n">
         <x:v>45909</x:v>
       </x:c>
       <x:c r="F33" s="9" t="str">
@@ -976,7 +982,7 @@
       <x:c r="D34" s="9" t="str">
         <x:v>Новосибирск</x:v>
       </x:c>
-      <x:c r="E34" s="9" t="n">
+      <x:c r="E34" s="10" t="n">
         <x:v>45662</x:v>
       </x:c>
       <x:c r="F34" s="9" t="str">
@@ -996,7 +1002,7 @@
       <x:c r="D35" s="9" t="str">
         <x:v>Новосибирск</x:v>
       </x:c>
-      <x:c r="E35" s="9" t="n">
+      <x:c r="E35" s="10" t="n">
         <x:v>45525</x:v>
       </x:c>
       <x:c r="F35" s="9" t="str">
@@ -1016,7 +1022,7 @@
       <x:c r="D36" s="9" t="str">
         <x:v>Новосибирск</x:v>
       </x:c>
-      <x:c r="E36" s="9" t="n">
+      <x:c r="E36" s="10" t="n">
         <x:v>45472</x:v>
       </x:c>
       <x:c r="F36" s="9" t="str">
@@ -1036,7 +1042,7 @@
       <x:c r="D37" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E37" s="9" t="n">
+      <x:c r="E37" s="10" t="n">
         <x:v>45408</x:v>
       </x:c>
       <x:c r="F37" s="9" t="str">
@@ -1056,7 +1062,7 @@
       <x:c r="D38" s="9" t="str">
         <x:v>Екатеринбург</x:v>
       </x:c>
-      <x:c r="E38" s="9" t="n">
+      <x:c r="E38" s="10" t="n">
         <x:v>45507</x:v>
       </x:c>
       <x:c r="F38" s="9" t="str">
@@ -1076,7 +1082,7 @@
       <x:c r="D39" s="9" t="str">
         <x:v>Новосибирск</x:v>
       </x:c>
-      <x:c r="E39" s="9" t="n">
+      <x:c r="E39" s="10" t="n">
         <x:v>45386</x:v>
       </x:c>
       <x:c r="F39" s="9" t="str">
@@ -1096,7 +1102,7 @@
       <x:c r="D40" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E40" s="9" t="n">
+      <x:c r="E40" s="10" t="n">
         <x:v>45876</x:v>
       </x:c>
       <x:c r="F40" s="9" t="str">
@@ -1116,7 +1122,7 @@
       <x:c r="D41" s="9" t="str">
         <x:v>Новосибирск</x:v>
       </x:c>
-      <x:c r="E41" s="9" t="n">
+      <x:c r="E41" s="10" t="n">
         <x:v>45875</x:v>
       </x:c>
       <x:c r="F41" s="9" t="str">
@@ -1136,7 +1142,7 @@
       <x:c r="D42" s="9" t="str">
         <x:v>Самара</x:v>
       </x:c>
-      <x:c r="E42" s="9" t="n">
+      <x:c r="E42" s="10" t="n">
         <x:v>45927</x:v>
       </x:c>
       <x:c r="F42" s="9" t="str">
@@ -1156,7 +1162,7 @@
       <x:c r="D43" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E43" s="9" t="n">
+      <x:c r="E43" s="10" t="n">
         <x:v>45295</x:v>
       </x:c>
       <x:c r="F43" s="9" t="str">
@@ -1176,7 +1182,7 @@
       <x:c r="D44" s="9" t="str">
         <x:v>Москва</x:v>
       </x:c>
-      <x:c r="E44" s="9" t="n">
+      <x:c r="E44" s="10" t="n">
         <x:v>45673</x:v>
       </x:c>
       <x:c r="F44" s="9" t="str">
@@ -1196,7 +1202,7 @@
       <x:c r="D45" s="9" t="str">
         <x:v>Екатеринбург</x:v>
       </x:c>
-      <x:c r="E45" s="9" t="n">
+      <x:c r="E45" s="10" t="n">
         <x:v>45723</x:v>
       </x:c>
       <x:c r="F45" s="9" t="str">
@@ -1216,7 +1222,7 @@
       <x:c r="D46" s="9" t="str">
         <x:v>Новосибирск</x:v>
       </x:c>
-      <x:c r="E46" s="9" t="n">
+      <x:c r="E46" s="10" t="n">
         <x:v>45554</x:v>
       </x:c>
       <x:c r="F46" s="9" t="str">
@@ -1236,7 +1242,7 @@
       <x:c r="D47" s="9" t="str">
         <x:v>Санкт-Петербург</x:v>
       </x:c>
-      <x:c r="E47" s="9" t="n">
+      <x:c r="E47" s="10" t="n">
         <x:v>45304</x:v>
       </x:c>
       <x:c r="F47" s="9" t="str">
@@ -1246,7 +1252,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d5889cccd9e4b95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R467b23a34e904106"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>